<commit_message>
Second version of Hat + add Pull-up on UART_RX of the control Board
</commit_message>
<xml_diff>
--- a/NPulse_v4/positions_connecteurs.xlsx
+++ b/NPulse_v4/positions_connecteurs.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/pCloud Drive/EPFL/NPulse/Transradial-Prosthesis-CTRL-HW/NPulse_v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66220D2-3E29-824F-9318-310F54470BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1B45C1-7603-1040-82A3-A602EFA1888A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17340" xr2:uid="{C7DDFD0C-C748-AA46-9479-7D0AC4BE6B94}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
   <si>
     <t>X</t>
   </si>
@@ -57,6 +57,12 @@
   </si>
   <si>
     <t>coin inférieur gauche</t>
+  </si>
+  <si>
+    <t>REF1</t>
+  </si>
+  <si>
+    <t>REF2</t>
   </si>
 </sst>
 </file>
@@ -230,9 +236,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -255,6 +258,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -591,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE6233D5-DAF1-854C-B5B5-CEBB80B9C173}">
-  <dimension ref="A2:J16"/>
+  <dimension ref="A2:N38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="10.83203125" style="1"/>
@@ -610,10 +616,10 @@
       <c r="F2" s="1">
         <v>6</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="2"/>
+      <c r="J2" s="10"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
@@ -699,101 +705,207 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4">
+      <c r="C10" s="2"/>
+      <c r="D10" s="3">
         <v>4</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>5</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <f>D3-$J$3</f>
         <v>10.610000000000014</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <f t="shared" ref="E11:F11" si="0">E3-$J$3</f>
         <v>21.620000000000005</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="7">
         <f t="shared" si="0"/>
         <v>32.620000000000005</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <f>D4-$J4</f>
         <v>-31.519999999999982</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <f t="shared" ref="E12:F12" si="1">E4-$J4</f>
         <v>-31.524999999999991</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="6">
         <f t="shared" si="1"/>
         <v>-31.534999999999982</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="C13" s="6"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="8"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="C14" s="6"/>
-      <c r="D14" s="7">
+      <c r="C14" s="5"/>
+      <c r="D14" s="6">
         <v>1</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="6">
         <v>2</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.2">
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <f>D7-$J$3</f>
         <v>7.0550000000000068</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <f t="shared" ref="E15:F15" si="2">E7-$J$3</f>
         <v>18.094999999999999</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="7">
         <f t="shared" si="2"/>
         <v>29.105000000000018</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <f>D8-$J4</f>
         <v>-11.519999999999982</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="9">
         <f t="shared" ref="E16:F16" si="3">E8-$J4</f>
         <v>-11.509999999999991</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="9">
         <f t="shared" si="3"/>
         <v>-11.509999999999991</v>
+      </c>
+    </row>
+    <row r="29" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="M29" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="I30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M30" s="1">
+        <v>148.97</v>
+      </c>
+      <c r="N30" s="1">
+        <v>122.17</v>
+      </c>
+    </row>
+    <row r="31" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="H31" s="1">
+        <v>1</v>
+      </c>
+      <c r="I31" s="1">
+        <v>184.65</v>
+      </c>
+      <c r="J31" s="1">
+        <v>121.38</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M31" s="1">
+        <v>155.01</v>
+      </c>
+      <c r="N31" s="1">
+        <v>136.01</v>
+      </c>
+    </row>
+    <row r="32" spans="8:14" x14ac:dyDescent="0.2">
+      <c r="H32" s="1">
+        <v>2</v>
+      </c>
+      <c r="I32" s="1">
+        <v>184.64</v>
+      </c>
+      <c r="J32" s="1">
+        <v>82.28</v>
+      </c>
+    </row>
+    <row r="33" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H33" s="1">
+        <v>3</v>
+      </c>
+      <c r="I33" s="1">
+        <v>149.82</v>
+      </c>
+      <c r="J33" s="1">
+        <v>82.34</v>
+      </c>
+    </row>
+    <row r="36" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H36" s="1">
+        <v>1</v>
+      </c>
+      <c r="I36" s="1">
+        <f>I31+$M$31-$M$30</f>
+        <v>190.68999999999997</v>
+      </c>
+      <c r="J36" s="1">
+        <f>J31+$N$31-$N$30</f>
+        <v>135.21999999999997</v>
+      </c>
+    </row>
+    <row r="37" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H37" s="1">
+        <v>2</v>
+      </c>
+      <c r="I37" s="1">
+        <f t="shared" ref="I37:I38" si="4">I32+$M$31-$M$30</f>
+        <v>190.67999999999998</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" ref="J37:J38" si="5">J32+$N$31-$N$30</f>
+        <v>96.11999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H38" s="1">
+        <v>3</v>
+      </c>
+      <c r="I38" s="1">
+        <f t="shared" si="4"/>
+        <v>155.85999999999999</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="5"/>
+        <v>96.179999999999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>